<commit_message>
this is final commit
</commit_message>
<xml_diff>
--- a/TestData/Test_Data.xlsx
+++ b/TestData/Test_Data.xlsx
@@ -385,7 +385,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -554,7 +554,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
+    <hyperlink ref="C3" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>